<commit_message>
Release updated Pareto workflow under MIT license
</commit_message>
<xml_diff>
--- a/output/csv/parameter_settings.xlsx
+++ b/output/csv/parameter_settings.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数设置" sheetId="1" r:id="R56cbf0dd75a840d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数设置" sheetId="1" r:id="Reb984347d57f4cc1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1410,7 +1410,7 @@
         <x:v>自动派生，请勿直接修改</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="55" t="str">
         <x:v>Stage A 与时间范围</x:v>
       </x:c>
@@ -1424,16 +1424,16 @@
         <x:v>相对值</x:v>
       </x:c>
       <x:c r="E35" s="45" t="str">
-        <x:v>Stage B 相对最短时间可增加的比例；0.02 表示 2%。</x:v>
+        <x:v>时间–振动 Pareto 前沿相对最短时间可增加的比例；0.02 表示 2%。</x:v>
       </x:c>
       <x:c r="F35" s="45" t="str">
-        <x:v>可用时间点增多，通常能获得更低振动。</x:v>
+        <x:v>整数时间候选点增多，Pareto 解更多，并通常能获得更低振动。</x:v>
       </x:c>
       <x:c r="G35" s="45" t="str">
-        <x:v>更接近严格最短时间，折中空间减少。</x:v>
+        <x:v>候选点减少且更接近严格最短时间。</x:v>
       </x:c>
       <x:c r="H35" s="47" t="str">
-        <x:v>建议按时间容许量修改</x:v>
+        <x:v>需要更多时间–振动 Pareto 解时提高</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -1632,16 +1632,16 @@
         <x:v>向量</x:v>
       </x:c>
       <x:c r="E43" s="45" t="str">
-        <x:v>Stage B 振动权重 lambda_vib 的扫描网格。</x:v>
+        <x:v>旧版“直线保持–振动”权重扫描参数；主流程的“时间–振动”Pareto 前沿不再使用。</x:v>
       </x:c>
       <x:c r="F43" s="45" t="str">
-        <x:v>增加权重点密度可得到更多 Pareto 解，但 NLP 次数增加。</x:v>
+        <x:v>对当前主流程无影响。</x:v>
       </x:c>
       <x:c r="G43" s="45" t="str">
-        <x:v>减少权重点可加快运行，但前沿更稀疏。</x:v>
+        <x:v>对当前主流程无影响。</x:v>
       </x:c>
       <x:c r="H43" s="47" t="str">
-        <x:v>需要更多 Pareto 解时修改</x:v>
+        <x:v>仅保留兼容性，不建议修改</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
@@ -1696,7 +1696,7 @@
         <x:v>仅研究双模态时开启</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="15" hidden="0" customHeight="1">
+    <x:row r="46" ht="36" hidden="0" customHeight="1">
       <x:c r="A46" s="44" t="str">
         <x:v>Pareto 与逐时间扫描</x:v>
       </x:c>
@@ -1710,19 +1710,19 @@
         <x:v>逻辑值</x:v>
       </x:c>
       <x:c r="E46" s="45" t="str">
-        <x:v>是否对 Nmin 到 Nmax 的每个整数时间求无抑制/有抑制成对解。</x:v>
+        <x:v>是否对 Nmin 到 Nmax 的每个整数时间求无抑制/有抑制成对解，并构建时间–振动 Pareto 前沿。</x:v>
       </x:c>
       <x:c r="F46" s="45" t="str">
-        <x:v>true 可得到完整逐时间对比，耗时显著增加。</x:v>
+        <x:v>true 生成主 Pareto 前沿。</x:v>
       </x:c>
       <x:c r="G46" s="45" t="str">
-        <x:v>false 跳过逐时间成对扫描。</x:v>
+        <x:v>false 无法生成主 Pareto 前沿。</x:v>
       </x:c>
       <x:c r="H46" s="50" t="str">
-        <x:v>需要完整对比时保持 true</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="15" hidden="0" customHeight="1">
+        <x:v>主流程必须保持 true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="24" hidden="0" customHeight="1">
       <x:c r="A47" s="44" t="str">
         <x:v>Pareto 与逐时间扫描</x:v>
       </x:c>
@@ -1736,16 +1736,16 @@
         <x:v>相对值</x:v>
       </x:c>
       <x:c r="E47" s="45" t="str">
-        <x:v>逐时间扫描中有抑制解采用的振动目标权重，范围 (0,1]。</x:v>
+        <x:v>固定时间下振动目标权重；时间–振动 Pareto 要求该值严格等于 1。</x:v>
       </x:c>
       <x:c r="F47" s="45" t="str">
-        <x:v>更强调完整振动目标。</x:v>
+        <x:v>不允许大于 1。</x:v>
       </x:c>
       <x:c r="G47" s="45" t="str">
-        <x:v>更保留直线保持目标，抑振强度可能下降。</x:v>
-      </x:c>
-      <x:c r="H47" s="47" t="str">
-        <x:v>建议按折中偏好修改</x:v>
+        <x:v>小于 1 会混入直线保持目标，程序将拒绝运行。</x:v>
+      </x:c>
+      <x:c r="H47" s="50" t="str">
+        <x:v>保持 1；用 cfg.objective.* 调整振动构成</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
@@ -3025,7 +3025,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4539fb721e25415e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd0a9305518b4355"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>